<commit_message>
Corrected typo in condition_occurrence_id
</commit_message>
<xml_diff>
--- a/config/MOHCCN to OMOP CDM Map v0.4.xlsx
+++ b/config/MOHCCN to OMOP CDM Map v0.4.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\serverfiles\projects\dhdp\mohccn-omop-etl\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\serverfiles\projects\python\mohccn-omop-etl\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42533032-F75B-4CD9-88A8-9EB2E4B5BDCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA7C6774-B1BA-48C1-9179-2717E0F7DC5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5959937F-EF1A-4EF7-9756-DEAA4796FC13}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4577" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4577" uniqueCount="730">
   <si>
     <t>mCODE Profile Name</t>
   </si>
@@ -1678,9 +1678,6 @@
   </si>
   <si>
     <t>observation.observation_id</t>
-  </si>
-  <si>
-    <t>condition_occurence_id</t>
   </si>
   <si>
     <t>condition_status_source_value</t>
@@ -2691,7 +2688,7 @@
         <v>236</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>237</v>
@@ -2700,7 +2697,7 @@
         <v>238</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="F1" s="6" t="s">
         <v>239</v>
@@ -2709,7 +2706,7 @@
         <v>240</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>241</v>
@@ -2718,7 +2715,7 @@
         <v>242</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>243</v>
@@ -2729,7 +2726,7 @@
         <v>244</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>245</v>
@@ -2753,7 +2750,7 @@
         <v>249</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -2773,7 +2770,7 @@
         <v>248</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
@@ -2801,7 +2798,7 @@
         <v>249</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -2827,15 +2824,15 @@
         <v>249</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D6" s="3" t="s">
+        <v>689</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>690</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>691</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>247</v>
@@ -2853,7 +2850,7 @@
         <v>249</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -2879,7 +2876,7 @@
         <v>249</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -2899,7 +2896,7 @@
         <v>248</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -2925,7 +2922,7 @@
         <v>249</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -2952,7 +2949,7 @@
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -2972,11 +2969,11 @@
         <v>9</v>
       </c>
       <c r="I11" s="4" t="str">
-        <f>$B$39</f>
+        <f t="shared" ref="I11:I19" si="0">$B$39</f>
         <v>OMOP Patient Person</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -2996,11 +2993,11 @@
         <v>9</v>
       </c>
       <c r="I12" s="4" t="str">
-        <f>$B$39</f>
+        <f t="shared" si="0"/>
         <v>OMOP Patient Person</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -3020,11 +3017,11 @@
         <v>9</v>
       </c>
       <c r="I13" s="4" t="str">
-        <f>$B$39</f>
+        <f t="shared" si="0"/>
         <v>OMOP Patient Person</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -3044,11 +3041,11 @@
         <v>9</v>
       </c>
       <c r="I14" s="4" t="str">
-        <f>$B$39</f>
+        <f t="shared" si="0"/>
         <v>OMOP Patient Person</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -3068,11 +3065,11 @@
         <v>9</v>
       </c>
       <c r="I15" s="4" t="str">
-        <f>$B$39</f>
+        <f t="shared" si="0"/>
         <v>OMOP Patient Person</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -3092,16 +3089,16 @@
         <v>9</v>
       </c>
       <c r="I16" s="4" t="str">
-        <f>$B$39</f>
+        <f t="shared" si="0"/>
         <v>OMOP Patient Person</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D17" s="3" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>262</v>
@@ -3116,11 +3113,11 @@
         <v>9</v>
       </c>
       <c r="I17" s="4" t="str">
-        <f>$B$39</f>
+        <f t="shared" si="0"/>
         <v>OMOP Patient Person</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -3140,11 +3137,11 @@
         <v>9</v>
       </c>
       <c r="I18" s="4" t="str">
-        <f>$B$39</f>
+        <f t="shared" si="0"/>
         <v>OMOP Patient Person</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
@@ -3164,11 +3161,11 @@
         <v>9</v>
       </c>
       <c r="I19" s="4" t="str">
-        <f>$B$39</f>
+        <f t="shared" si="0"/>
         <v>OMOP Patient Person</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -3179,7 +3176,7 @@
         <v>264</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>39</v>
@@ -3200,7 +3197,7 @@
         <v>264</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>84</v>
@@ -3221,7 +3218,7 @@
         <v>264</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>132</v>
@@ -3242,7 +3239,7 @@
         <v>264</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>200</v>
@@ -3263,7 +3260,7 @@
         <v>265</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>39</v>
@@ -3289,7 +3286,7 @@
         <v>265</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>84</v>
@@ -3315,7 +3312,7 @@
         <v>265</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>132</v>
@@ -3341,7 +3338,7 @@
         <v>265</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>200</v>
@@ -3350,30 +3347,30 @@
         <v>201</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>267</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>248</v>
@@ -3385,10 +3382,10 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D29" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>269</v>
@@ -3400,15 +3397,15 @@
         <v>248</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D30" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>247</v>
@@ -3420,15 +3417,15 @@
         <v>248</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D31" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>247</v>
@@ -3440,15 +3437,15 @@
         <v>248</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D32" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>247</v>
@@ -3465,10 +3462,10 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D33" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>247</v>
@@ -3480,22 +3477,22 @@
         <v>248</v>
       </c>
       <c r="I33" s="15" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="4" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>16</v>
@@ -3506,13 +3503,13 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D35" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>16</v>
@@ -3523,13 +3520,13 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D36" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>16</v>
@@ -3540,13 +3537,13 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D37" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>16</v>
@@ -3558,10 +3555,10 @@
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B38" s="3"/>
       <c r="D38" s="3" t="s">
+        <v>709</v>
+      </c>
+      <c r="E38" s="3" t="s">
         <v>710</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>711</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>269</v>
@@ -3573,16 +3570,16 @@
         <v>248</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="4" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>270</v>
@@ -3600,7 +3597,7 @@
         <v>9</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
@@ -3617,10 +3614,10 @@
         <v>248</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
@@ -3643,7 +3640,7 @@
         <v>274</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="L41" s="3" t="s">
         <v>275</v>
@@ -3683,7 +3680,7 @@
         <v>31</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -3703,7 +3700,7 @@
         <v>31</v>
       </c>
       <c r="K44" s="3" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
@@ -3723,12 +3720,12 @@
         <v>31</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E46" s="3" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>269</v>
@@ -3740,12 +3737,12 @@
         <v>248</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E47" s="3" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>269</v>
@@ -3757,12 +3754,12 @@
         <v>248</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B48" s="4" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>245</v>
@@ -3780,7 +3777,7 @@
         <v>9</v>
       </c>
       <c r="K48" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
@@ -3803,7 +3800,7 @@
         <v>289</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.25">
@@ -3823,7 +3820,7 @@
         <v>21</v>
       </c>
       <c r="K50" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
@@ -3845,7 +3842,7 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B52" s="4" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>294</v>
@@ -3870,7 +3867,7 @@
       </c>
       <c r="K52" s="2"/>
       <c r="L52" s="3" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.25">
@@ -3890,7 +3887,7 @@
         <v>33</v>
       </c>
       <c r="K53" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.25">
@@ -3929,7 +3926,7 @@
     </row>
     <row r="56" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B56" s="4" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="E56" s="3" t="s">
         <v>303</v>
@@ -3965,19 +3962,19 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>84</v>
@@ -3986,7 +3983,7 @@
         <v>43</v>
       </c>
       <c r="K59" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
@@ -4007,7 +4004,7 @@
         <v>43</v>
       </c>
       <c r="K60" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
@@ -4030,7 +4027,7 @@
         <v>308</v>
       </c>
       <c r="K61" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.25">
@@ -4068,7 +4065,7 @@
       </c>
       <c r="I63" s="3"/>
       <c r="K63" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
@@ -4097,7 +4094,7 @@
     </row>
     <row r="65" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B65" s="4" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>251</v>
@@ -4115,7 +4112,7 @@
         <v>43</v>
       </c>
       <c r="K65" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="66" spans="2:12" x14ac:dyDescent="0.25">
@@ -4176,7 +4173,7 @@
         <v>308</v>
       </c>
       <c r="K68" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="69" spans="2:12" x14ac:dyDescent="0.25">
@@ -4210,7 +4207,7 @@
         <v>248</v>
       </c>
       <c r="I70" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="71" spans="2:12" x14ac:dyDescent="0.25">
@@ -4227,12 +4224,12 @@
         <v>248</v>
       </c>
       <c r="I71" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="72" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B72" s="4" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>325</v>
@@ -4254,7 +4251,7 @@
         <v>OMOP Primary Dx Episode</v>
       </c>
       <c r="K72" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="73" spans="2:12" x14ac:dyDescent="0.25">
@@ -4275,7 +4272,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K73" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="74" spans="2:12" x14ac:dyDescent="0.25">
@@ -4298,12 +4295,12 @@
         <v>267</v>
       </c>
       <c r="L74" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="75" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B75" s="4" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>255</v>
@@ -4321,7 +4318,7 @@
         <v>43</v>
       </c>
       <c r="K75" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="76" spans="2:12" x14ac:dyDescent="0.25">
@@ -4361,7 +4358,7 @@
         <v>248</v>
       </c>
       <c r="I77" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="78" spans="2:12" x14ac:dyDescent="0.25">
@@ -4382,7 +4379,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K78" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="79" spans="2:12" x14ac:dyDescent="0.25">
@@ -4405,7 +4402,7 @@
         <v>267</v>
       </c>
       <c r="L79" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="80" spans="2:12" x14ac:dyDescent="0.25">
@@ -4444,7 +4441,7 @@
     </row>
     <row r="82" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B82" s="4" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>255</v>
@@ -4462,7 +4459,7 @@
         <v>43</v>
       </c>
       <c r="K82" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="83" spans="2:12" x14ac:dyDescent="0.25">
@@ -4485,7 +4482,7 @@
         <v>335</v>
       </c>
       <c r="L83" s="3" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="84" spans="2:12" x14ac:dyDescent="0.25">
@@ -4502,7 +4499,7 @@
         <v>248</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="85" spans="2:12" x14ac:dyDescent="0.25">
@@ -4523,7 +4520,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K85" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.25">
@@ -4546,7 +4543,7 @@
         <v>267</v>
       </c>
       <c r="L86" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="87" spans="2:12" x14ac:dyDescent="0.25">
@@ -4566,7 +4563,7 @@
         <v>94</v>
       </c>
       <c r="K87" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="88" spans="2:12" x14ac:dyDescent="0.25">
@@ -4588,7 +4585,7 @@
     </row>
     <row r="89" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B89" s="4" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>245</v>
@@ -4606,7 +4603,7 @@
         <v>43</v>
       </c>
       <c r="K89" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="90" spans="2:12" x14ac:dyDescent="0.25">
@@ -4646,7 +4643,7 @@
         <v>248</v>
       </c>
       <c r="I91" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="92" spans="2:12" x14ac:dyDescent="0.25">
@@ -4666,7 +4663,7 @@
         <v>91</v>
       </c>
       <c r="K92" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="93" spans="2:12" x14ac:dyDescent="0.25">
@@ -4704,7 +4701,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K94" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="95" spans="2:12" x14ac:dyDescent="0.25">
@@ -4727,12 +4724,12 @@
         <v>267</v>
       </c>
       <c r="L95" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="96" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B96" s="4" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>255</v>
@@ -4750,7 +4747,7 @@
         <v>43</v>
       </c>
       <c r="K96" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="97" spans="2:12" x14ac:dyDescent="0.25">
@@ -4767,13 +4764,13 @@
         <v>248</v>
       </c>
       <c r="I97" s="4" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="J97" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L97" s="3" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="98" spans="2:12" x14ac:dyDescent="0.25">
@@ -4790,7 +4787,7 @@
         <v>248</v>
       </c>
       <c r="I98" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="99" spans="2:12" x14ac:dyDescent="0.25">
@@ -4811,7 +4808,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K99" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="100" spans="2:12" x14ac:dyDescent="0.25">
@@ -4834,7 +4831,7 @@
         <v>267</v>
       </c>
       <c r="L100" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="101" spans="2:12" x14ac:dyDescent="0.25">
@@ -4854,7 +4851,7 @@
         <v>114</v>
       </c>
       <c r="K101" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="102" spans="2:12" x14ac:dyDescent="0.25">
@@ -4876,7 +4873,7 @@
     </row>
     <row r="103" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B103" s="4" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>255</v>
@@ -4894,7 +4891,7 @@
         <v>43</v>
       </c>
       <c r="K103" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="104" spans="2:12" x14ac:dyDescent="0.25">
@@ -4911,13 +4908,13 @@
         <v>248</v>
       </c>
       <c r="I104" s="4" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="J104" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L104" s="3" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="105" spans="2:12" x14ac:dyDescent="0.25">
@@ -4934,7 +4931,7 @@
         <v>248</v>
       </c>
       <c r="I105" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="106" spans="2:12" x14ac:dyDescent="0.25">
@@ -4955,7 +4952,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K106" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="107" spans="2:12" x14ac:dyDescent="0.25">
@@ -4978,7 +4975,7 @@
         <v>267</v>
       </c>
       <c r="L107" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="108" spans="2:12" x14ac:dyDescent="0.25">
@@ -4998,7 +4995,7 @@
         <v>119</v>
       </c>
       <c r="K108" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="109" spans="2:12" x14ac:dyDescent="0.25">
@@ -5020,7 +5017,7 @@
     </row>
     <row r="110" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B110" s="4" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>255</v>
@@ -5038,7 +5035,7 @@
         <v>43</v>
       </c>
       <c r="K110" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="111" spans="2:12" x14ac:dyDescent="0.25">
@@ -5055,13 +5052,13 @@
         <v>248</v>
       </c>
       <c r="I111" s="4" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="J111" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L111" s="3" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="112" spans="2:12" x14ac:dyDescent="0.25">
@@ -5078,7 +5075,7 @@
         <v>248</v>
       </c>
       <c r="I112" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="113" spans="2:12" x14ac:dyDescent="0.25">
@@ -5099,7 +5096,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K113" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="114" spans="2:12" x14ac:dyDescent="0.25">
@@ -5122,7 +5119,7 @@
         <v>267</v>
       </c>
       <c r="L114" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="115" spans="2:12" x14ac:dyDescent="0.25">
@@ -5142,7 +5139,7 @@
         <v>124</v>
       </c>
       <c r="K115" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="116" spans="2:12" x14ac:dyDescent="0.25">
@@ -5164,7 +5161,7 @@
     </row>
     <row r="117" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B117" s="4" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="D117" s="3" t="s">
         <v>255</v>
@@ -5182,7 +5179,7 @@
         <v>43</v>
       </c>
       <c r="K117" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="118" spans="2:12" x14ac:dyDescent="0.25">
@@ -5202,7 +5199,7 @@
         <v>98</v>
       </c>
       <c r="K118" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="119" spans="2:12" x14ac:dyDescent="0.25">
@@ -5236,7 +5233,7 @@
         <v>248</v>
       </c>
       <c r="I120" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="121" spans="2:12" x14ac:dyDescent="0.25">
@@ -5277,7 +5274,7 @@
         <v>267</v>
       </c>
       <c r="L122" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="123" spans="2:12" x14ac:dyDescent="0.25">
@@ -5316,7 +5313,7 @@
     </row>
     <row r="125" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B125" s="4" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>255</v>
@@ -5334,7 +5331,7 @@
         <v>43</v>
       </c>
       <c r="K125" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="126" spans="2:12" x14ac:dyDescent="0.25">
@@ -5351,13 +5348,13 @@
         <v>248</v>
       </c>
       <c r="I126" s="4" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="J126" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L126" s="3" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="127" spans="2:12" x14ac:dyDescent="0.25">
@@ -5374,7 +5371,7 @@
         <v>248</v>
       </c>
       <c r="I127" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="128" spans="2:12" x14ac:dyDescent="0.25">
@@ -5395,7 +5392,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K128" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="129" spans="2:12" x14ac:dyDescent="0.25">
@@ -5418,7 +5415,7 @@
         <v>267</v>
       </c>
       <c r="L129" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="130" spans="2:12" x14ac:dyDescent="0.25">
@@ -5438,7 +5435,7 @@
         <v>127</v>
       </c>
       <c r="K130" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="131" spans="2:12" x14ac:dyDescent="0.25">
@@ -5460,7 +5457,7 @@
     </row>
     <row r="132" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B132" s="4" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="D132" s="3" t="s">
         <v>255</v>
@@ -5478,7 +5475,7 @@
         <v>43</v>
       </c>
       <c r="K132" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="133" spans="2:12" x14ac:dyDescent="0.25">
@@ -5495,13 +5492,13 @@
         <v>248</v>
       </c>
       <c r="I133" s="4" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="J133" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L133" s="3" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="134" spans="2:12" x14ac:dyDescent="0.25">
@@ -5518,7 +5515,7 @@
         <v>248</v>
       </c>
       <c r="I134" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="135" spans="2:12" x14ac:dyDescent="0.25">
@@ -5539,7 +5536,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K135" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="136" spans="2:12" x14ac:dyDescent="0.25">
@@ -5562,7 +5559,7 @@
         <v>267</v>
       </c>
       <c r="L136" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="137" spans="2:12" x14ac:dyDescent="0.25">
@@ -5582,7 +5579,7 @@
         <v>129</v>
       </c>
       <c r="K137" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="138" spans="2:12" x14ac:dyDescent="0.25">
@@ -5604,7 +5601,7 @@
     </row>
     <row r="139" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B139" s="4" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>255</v>
@@ -5622,7 +5619,7 @@
         <v>43</v>
       </c>
       <c r="K139" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="140" spans="2:12" x14ac:dyDescent="0.25">
@@ -5639,13 +5636,13 @@
         <v>248</v>
       </c>
       <c r="I140" s="4" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="J140" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L140" s="3" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="141" spans="2:12" x14ac:dyDescent="0.25">
@@ -5662,7 +5659,7 @@
         <v>248</v>
       </c>
       <c r="I141" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="142" spans="2:12" x14ac:dyDescent="0.25">
@@ -5683,7 +5680,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K142" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="143" spans="2:12" x14ac:dyDescent="0.25">
@@ -5706,7 +5703,7 @@
         <v>267</v>
       </c>
       <c r="L143" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="144" spans="2:12" x14ac:dyDescent="0.25">
@@ -5726,7 +5723,7 @@
         <v>131</v>
       </c>
       <c r="K144" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="145" spans="1:12" x14ac:dyDescent="0.25">
@@ -5748,7 +5745,7 @@
     </row>
     <row r="146" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B146" s="4" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="D146" s="3" t="s">
         <v>255</v>
@@ -5766,7 +5763,7 @@
         <v>43</v>
       </c>
       <c r="K146" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="147" spans="1:12" x14ac:dyDescent="0.25">
@@ -5786,7 +5783,7 @@
         <v>102</v>
       </c>
       <c r="K147" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="148" spans="1:12" x14ac:dyDescent="0.25">
@@ -5820,7 +5817,7 @@
         <v>248</v>
       </c>
       <c r="I149" s="3" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="150" spans="1:12" x14ac:dyDescent="0.25">
@@ -5841,7 +5838,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K150" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="151" spans="1:12" x14ac:dyDescent="0.25">
@@ -5864,7 +5861,7 @@
         <v>267</v>
       </c>
       <c r="L151" s="3" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="152" spans="1:12" x14ac:dyDescent="0.25">
@@ -5886,7 +5883,7 @@
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C153" s="3" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="E153" s="3" t="s">
         <v>293</v>
@@ -5903,19 +5900,19 @@
     </row>
     <row r="154" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A154" s="6" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E154" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F154" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G154" s="3" t="s">
         <v>132</v>
@@ -5924,18 +5921,18 @@
         <v>44</v>
       </c>
       <c r="K154" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="155" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D155" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E155" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F155" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G155" s="3" t="s">
         <v>132</v>
@@ -5944,18 +5941,18 @@
         <v>135</v>
       </c>
       <c r="K155" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D156" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E156" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F156" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G156" s="3" t="s">
         <v>132</v>
@@ -5983,7 +5980,7 @@
         <v>44</v>
       </c>
       <c r="K157" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.25">
@@ -6060,7 +6057,7 @@
         <v>135</v>
       </c>
       <c r="K161" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="162" spans="2:12" x14ac:dyDescent="0.25">
@@ -6099,7 +6096,7 @@
     </row>
     <row r="164" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B164" s="4" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="D164" s="3" t="s">
         <v>245</v>
@@ -6117,7 +6114,7 @@
         <v>44</v>
       </c>
       <c r="K164" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="165" spans="2:12" x14ac:dyDescent="0.25">
@@ -6134,13 +6131,13 @@
         <v>248</v>
       </c>
       <c r="I165" s="4" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="J165" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L165" s="3" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="166" spans="2:12" x14ac:dyDescent="0.25">
@@ -6157,7 +6154,7 @@
         <v>135</v>
       </c>
       <c r="K166" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="167" spans="2:12" x14ac:dyDescent="0.25">
@@ -6178,7 +6175,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K167" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="168" spans="2:12" x14ac:dyDescent="0.25">
@@ -6221,7 +6218,7 @@
         <v>137</v>
       </c>
       <c r="K169" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="170" spans="2:12" x14ac:dyDescent="0.25">
@@ -6243,7 +6240,7 @@
     </row>
     <row r="171" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B171" s="4" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D171" s="3" t="s">
         <v>245</v>
@@ -6261,7 +6258,7 @@
         <v>44</v>
       </c>
       <c r="K171" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="172" spans="2:12" x14ac:dyDescent="0.25">
@@ -6301,10 +6298,10 @@
         <v>132</v>
       </c>
       <c r="H173" s="7" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="K173" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="174" spans="2:12" x14ac:dyDescent="0.25">
@@ -6321,7 +6318,7 @@
         <v>132</v>
       </c>
       <c r="H174" s="7" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="175" spans="2:12" x14ac:dyDescent="0.25">
@@ -6338,7 +6335,7 @@
         <v>135</v>
       </c>
       <c r="K175" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="176" spans="2:12" x14ac:dyDescent="0.25">
@@ -6359,7 +6356,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K176" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="177" spans="1:12" x14ac:dyDescent="0.25">
@@ -6421,10 +6418,10 @@
     </row>
     <row r="180" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A180" s="6" t="s">
+        <v>723</v>
+      </c>
+      <c r="B180" s="4" t="s">
         <v>724</v>
-      </c>
-      <c r="B180" s="4" t="s">
-        <v>725</v>
       </c>
       <c r="D180" s="3" t="s">
         <v>258</v>
@@ -6433,7 +6430,7 @@
         <v>370</v>
       </c>
       <c r="F180" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G180" s="3" t="s">
         <v>132</v>
@@ -6442,7 +6439,7 @@
         <v>44</v>
       </c>
       <c r="K180" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="181" spans="1:12" x14ac:dyDescent="0.25">
@@ -6459,7 +6456,7 @@
         <v>248</v>
       </c>
       <c r="I181" s="4" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="182" spans="1:12" x14ac:dyDescent="0.25">
@@ -6470,7 +6467,7 @@
         <v>373</v>
       </c>
       <c r="F182" s="3" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="G182" s="3" t="s">
         <v>248</v>
@@ -6493,10 +6490,10 @@
         <v>248</v>
       </c>
       <c r="I183" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K183" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="184" spans="1:12" x14ac:dyDescent="0.25">
@@ -6516,7 +6513,7 @@
         <v>248</v>
       </c>
       <c r="I184" s="4" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="185" spans="1:12" x14ac:dyDescent="0.25">
@@ -6536,12 +6533,12 @@
         <v>248</v>
       </c>
       <c r="I185" s="4" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="186" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B186" s="4" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="D186" s="3" t="s">
         <v>325</v>
@@ -6563,7 +6560,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K186" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="187" spans="1:12" x14ac:dyDescent="0.25">
@@ -6584,7 +6581,7 @@
         <v>OMOP Treatment Episode Procedure Occurrence</v>
       </c>
       <c r="K187" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="188" spans="1:12" x14ac:dyDescent="0.25">
@@ -6612,10 +6609,10 @@
     </row>
     <row r="189" spans="1:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="A189" s="6" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="D189" s="3" t="s">
         <v>251</v>
@@ -6634,7 +6631,7 @@
       </c>
       <c r="I189" s="3"/>
       <c r="K189" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="190" spans="1:12" x14ac:dyDescent="0.25">
@@ -6692,7 +6689,7 @@
       </c>
       <c r="I192" s="6"/>
       <c r="K192" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="193" spans="2:12" x14ac:dyDescent="0.25">
@@ -6709,7 +6706,7 @@
         <v>146</v>
       </c>
       <c r="K193" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="194" spans="2:12" x14ac:dyDescent="0.25">
@@ -6728,7 +6725,7 @@
     </row>
     <row r="195" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B195" s="4" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="D195" s="3" t="s">
         <v>325</v>
@@ -6750,7 +6747,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K195" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="196" spans="2:12" x14ac:dyDescent="0.25">
@@ -6771,7 +6768,7 @@
         <v>OMOP Systemic Therapy Episode</v>
       </c>
       <c r="K196" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="197" spans="2:12" x14ac:dyDescent="0.25">
@@ -6799,7 +6796,7 @@
     </row>
     <row r="198" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B198" s="4" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="D198" s="3" t="s">
         <v>258</v>
@@ -6818,7 +6815,7 @@
       </c>
       <c r="I198" s="3"/>
       <c r="K198" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="199" spans="2:12" x14ac:dyDescent="0.25">
@@ -6838,7 +6835,7 @@
         <v>145</v>
       </c>
       <c r="K199" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="200" spans="2:12" x14ac:dyDescent="0.25">
@@ -6872,7 +6869,7 @@
         <v>146</v>
       </c>
       <c r="K201" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="202" spans="2:12" x14ac:dyDescent="0.25">
@@ -6894,7 +6891,7 @@
     </row>
     <row r="203" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B203" s="4" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="D203" s="3" t="s">
         <v>325</v>
@@ -6916,7 +6913,7 @@
         <v>OMOP Systemic Therapy Episode</v>
       </c>
       <c r="K203" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="204" spans="2:12" x14ac:dyDescent="0.25">
@@ -6937,7 +6934,7 @@
         <v>OMOP Systemic Therapy Procedure</v>
       </c>
       <c r="K204" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="205" spans="2:12" x14ac:dyDescent="0.25">
@@ -6965,13 +6962,13 @@
     </row>
     <row r="206" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B206" s="4" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="D206" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E206" s="3" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="F206" s="3" t="s">
         <v>269</v>
@@ -6984,7 +6981,7 @@
       </c>
       <c r="I206" s="11"/>
       <c r="K206" s="3" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="207" spans="2:12" x14ac:dyDescent="0.25">
@@ -7005,7 +7002,7 @@
         <v>44</v>
       </c>
       <c r="K207" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="208" spans="2:12" x14ac:dyDescent="0.25">
@@ -7045,10 +7042,10 @@
         <v>149</v>
       </c>
       <c r="J209" s="3" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="K209" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="210" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
@@ -7059,7 +7056,7 @@
         <v>407</v>
       </c>
       <c r="F210" s="3" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G210" s="3" t="s">
         <v>141</v>
@@ -7085,7 +7082,7 @@
         <v>146</v>
       </c>
       <c r="K211" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="212" spans="2:12" x14ac:dyDescent="0.25">
@@ -7105,7 +7102,7 @@
         <v>147</v>
       </c>
       <c r="K212" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="213" spans="2:12" x14ac:dyDescent="0.25">
@@ -7144,7 +7141,7 @@
     </row>
     <row r="215" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B215" s="4" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="D215" s="3" t="s">
         <v>325</v>
@@ -7166,7 +7163,7 @@
         <v>OMOP Systemic Therapy Episode</v>
       </c>
       <c r="K215" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="216" spans="2:12" x14ac:dyDescent="0.25">
@@ -7187,7 +7184,7 @@
         <v>OMOP Systemic Therapy Dose Given Drug Exposure</v>
       </c>
       <c r="K216" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="217" spans="2:12" x14ac:dyDescent="0.25">
@@ -7215,7 +7212,7 @@
     </row>
     <row r="218" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B218" s="4" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="D218" s="3" t="s">
         <v>399</v>
@@ -7233,7 +7230,7 @@
         <v>44</v>
       </c>
       <c r="K218" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="219" spans="2:12" x14ac:dyDescent="0.25">
@@ -7273,10 +7270,10 @@
         <v>149</v>
       </c>
       <c r="J220" s="3" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="K220" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="221" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
@@ -7287,7 +7284,7 @@
         <v>407</v>
       </c>
       <c r="F221" s="3" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G221" s="3" t="s">
         <v>141</v>
@@ -7313,7 +7310,7 @@
         <v>146</v>
       </c>
       <c r="K222" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="223" spans="2:12" x14ac:dyDescent="0.25">
@@ -7333,7 +7330,7 @@
         <v>147</v>
       </c>
       <c r="K223" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="224" spans="2:12" x14ac:dyDescent="0.25">
@@ -7372,7 +7369,7 @@
     </row>
     <row r="226" spans="1:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B226" s="4" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="D226" s="3" t="s">
         <v>325</v>
@@ -7394,7 +7391,7 @@
         <v>OMOP Systemic Therapy Episode</v>
       </c>
       <c r="K226" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="227" spans="1:12" x14ac:dyDescent="0.25">
@@ -7415,7 +7412,7 @@
         <v>OMOP Systemic Therapy Dose Prescribed Drug Exposure</v>
       </c>
       <c r="K227" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="228" spans="1:12" x14ac:dyDescent="0.25">
@@ -7443,7 +7440,7 @@
     </row>
     <row r="229" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B229" s="4" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="G229" s="3" t="s">
         <v>141</v>
@@ -7454,10 +7451,10 @@
     </row>
     <row r="230" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A230" s="6" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="B230" s="4" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D230" s="3" t="s">
         <v>251</v>
@@ -7475,7 +7472,7 @@
         <v>44</v>
       </c>
       <c r="K230" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="231" spans="1:12" x14ac:dyDescent="0.25">
@@ -7533,7 +7530,7 @@
       </c>
       <c r="I233" s="6"/>
       <c r="K233" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="234" spans="1:12" x14ac:dyDescent="0.25">
@@ -7550,15 +7547,15 @@
         <v>248</v>
       </c>
       <c r="I234" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K234" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="235" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B235" s="4" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="D235" s="3" t="s">
         <v>325</v>
@@ -7580,7 +7577,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K235" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="236" spans="1:12" x14ac:dyDescent="0.25">
@@ -7601,7 +7598,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K236" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="237" spans="1:12" x14ac:dyDescent="0.25">
@@ -7629,7 +7626,7 @@
     </row>
     <row r="238" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B238" s="4" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D238" s="3" t="s">
         <v>258</v>
@@ -7647,7 +7644,7 @@
         <v>44</v>
       </c>
       <c r="K238" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="239" spans="1:12" x14ac:dyDescent="0.25">
@@ -7667,7 +7664,7 @@
         <v>162</v>
       </c>
       <c r="K239" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="240" spans="1:12" x14ac:dyDescent="0.25">
@@ -7701,10 +7698,10 @@
         <v>248</v>
       </c>
       <c r="I241" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K241" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="242" spans="2:12" x14ac:dyDescent="0.25">
@@ -7745,7 +7742,7 @@
     </row>
     <row r="244" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B244" s="4" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D244" s="3" t="s">
         <v>325</v>
@@ -7767,7 +7764,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K244" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="245" spans="2:12" x14ac:dyDescent="0.25">
@@ -7788,7 +7785,7 @@
         <v>OMOP Radiation Procedure</v>
       </c>
       <c r="K245" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="246" spans="2:12" x14ac:dyDescent="0.25">
@@ -7816,7 +7813,7 @@
     </row>
     <row r="247" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B247" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D247" s="3" t="s">
         <v>255</v>
@@ -7834,7 +7831,7 @@
         <v>44</v>
       </c>
       <c r="K247" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="248" spans="2:12" x14ac:dyDescent="0.25">
@@ -7874,10 +7871,10 @@
         <v>248</v>
       </c>
       <c r="I249" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K249" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="250" spans="2:12" x14ac:dyDescent="0.25">
@@ -7898,7 +7895,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K250" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="251" spans="2:12" x14ac:dyDescent="0.25">
@@ -7941,7 +7938,7 @@
         <v>167</v>
       </c>
       <c r="K252" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="253" spans="2:12" x14ac:dyDescent="0.25">
@@ -7972,7 +7969,7 @@
     </row>
     <row r="254" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B254" s="4" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D254" s="3" t="s">
         <v>255</v>
@@ -7990,7 +7987,7 @@
         <v>44</v>
       </c>
       <c r="K254" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="255" spans="2:12" x14ac:dyDescent="0.25">
@@ -8028,10 +8025,10 @@
         <v>248</v>
       </c>
       <c r="I256" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K256" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="257" spans="2:12" x14ac:dyDescent="0.25">
@@ -8052,7 +8049,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K257" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="258" spans="2:12" x14ac:dyDescent="0.25">
@@ -8095,12 +8092,12 @@
         <v>165</v>
       </c>
       <c r="K259" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="260" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B260" s="4" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="D260" s="3" t="s">
         <v>245</v>
@@ -8118,7 +8115,7 @@
         <v>44</v>
       </c>
       <c r="K260" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="261" spans="2:12" x14ac:dyDescent="0.25">
@@ -8158,10 +8155,10 @@
         <v>248</v>
       </c>
       <c r="I262" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K262" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="263" spans="2:12" x14ac:dyDescent="0.25">
@@ -8182,7 +8179,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K263" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="264" spans="2:12" x14ac:dyDescent="0.25">
@@ -8225,7 +8222,7 @@
         <v>170</v>
       </c>
       <c r="K265" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="266" spans="2:12" x14ac:dyDescent="0.25">
@@ -8247,7 +8244,7 @@
     </row>
     <row r="267" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B267" s="4" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="D267" s="3" t="s">
         <v>258</v>
@@ -8265,7 +8262,7 @@
         <v>44</v>
       </c>
       <c r="K267" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="268" spans="2:12" x14ac:dyDescent="0.25">
@@ -8305,10 +8302,10 @@
         <v>248</v>
       </c>
       <c r="I269" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K269" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="270" spans="2:12" x14ac:dyDescent="0.25">
@@ -8325,7 +8322,7 @@
         <v>171</v>
       </c>
       <c r="K270" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="271" spans="2:12" x14ac:dyDescent="0.25">
@@ -8344,7 +8341,7 @@
     </row>
     <row r="272" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B272" s="4" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D272" s="3" t="s">
         <v>325</v>
@@ -8366,7 +8363,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K272" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="273" spans="1:12" x14ac:dyDescent="0.25">
@@ -8387,7 +8384,7 @@
         <v>OMOP Radiation Boost Procedure</v>
       </c>
       <c r="K273" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="274" spans="1:12" x14ac:dyDescent="0.25">
@@ -8415,19 +8412,19 @@
     </row>
     <row r="275" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A275" s="6" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="B275" s="4" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="D275" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E275" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F275" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G275" s="3" t="s">
         <v>179</v>
@@ -8453,7 +8450,7 @@
         <v>44</v>
       </c>
       <c r="K276" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="277" spans="1:12" x14ac:dyDescent="0.25">
@@ -8511,10 +8508,10 @@
       </c>
       <c r="I279" s="6"/>
       <c r="J279" s="3" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="K279" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="280" spans="1:12" x14ac:dyDescent="0.25">
@@ -8531,15 +8528,15 @@
         <v>248</v>
       </c>
       <c r="I280" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K280" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="281" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B281" s="4" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D281" s="3" t="s">
         <v>325</v>
@@ -8561,7 +8558,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K281" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="282" spans="1:12" x14ac:dyDescent="0.25">
@@ -8582,7 +8579,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K282" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="283" spans="1:12" x14ac:dyDescent="0.25">
@@ -8610,7 +8607,7 @@
     </row>
     <row r="284" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B284" s="4" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D284" s="3" t="s">
         <v>258</v>
@@ -8628,7 +8625,7 @@
         <v>44</v>
       </c>
       <c r="K284" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="285" spans="1:12" x14ac:dyDescent="0.25">
@@ -8649,10 +8646,10 @@
       </c>
       <c r="I285" s="6"/>
       <c r="J285" s="3" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="K285" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="286" spans="1:12" ht="40.5" x14ac:dyDescent="0.25">
@@ -8663,7 +8660,7 @@
         <v>373</v>
       </c>
       <c r="F286" s="3" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G286" s="3" t="s">
         <v>179</v>
@@ -8686,15 +8683,15 @@
         <v>248</v>
       </c>
       <c r="I287" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K287" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="288" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B288" s="4" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="D288" s="3" t="s">
         <v>325</v>
@@ -8716,7 +8713,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K288" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="289" spans="2:12" x14ac:dyDescent="0.25">
@@ -8737,7 +8734,7 @@
         <v>OMOP Surgery Procedure</v>
       </c>
       <c r="K289" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="290" spans="2:12" x14ac:dyDescent="0.25">
@@ -8765,7 +8762,7 @@
     </row>
     <row r="291" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B291" s="4" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="D291" s="3" t="s">
         <v>255</v>
@@ -8783,7 +8780,7 @@
         <v>44</v>
       </c>
       <c r="K291" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="292" spans="2:12" x14ac:dyDescent="0.25">
@@ -8818,10 +8815,10 @@
         <v>248</v>
       </c>
       <c r="I293" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K293" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="294" spans="2:12" x14ac:dyDescent="0.25">
@@ -8842,7 +8839,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K294" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="295" spans="2:12" x14ac:dyDescent="0.25">
@@ -8885,7 +8882,7 @@
         <v>188</v>
       </c>
       <c r="K296" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="297" spans="2:12" x14ac:dyDescent="0.25">
@@ -8913,7 +8910,7 @@
     </row>
     <row r="298" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B298" s="4" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D298" s="3" t="s">
         <v>255</v>
@@ -8931,7 +8928,7 @@
         <v>44</v>
       </c>
       <c r="K298" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="299" spans="2:12" x14ac:dyDescent="0.25">
@@ -8966,10 +8963,10 @@
         <v>248</v>
       </c>
       <c r="I300" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K300" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="301" spans="2:12" x14ac:dyDescent="0.25">
@@ -8990,7 +8987,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K301" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="302" spans="2:12" x14ac:dyDescent="0.25">
@@ -9033,7 +9030,7 @@
         <v>190</v>
       </c>
       <c r="K303" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="304" spans="2:12" x14ac:dyDescent="0.25">
@@ -9061,7 +9058,7 @@
     </row>
     <row r="305" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B305" s="4" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="D305" s="3" t="s">
         <v>255</v>
@@ -9079,7 +9076,7 @@
         <v>44</v>
       </c>
       <c r="K305" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="306" spans="2:12" x14ac:dyDescent="0.25">
@@ -9114,10 +9111,10 @@
         <v>248</v>
       </c>
       <c r="I307" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K307" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="308" spans="2:12" x14ac:dyDescent="0.25">
@@ -9138,7 +9135,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K308" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="309" spans="2:12" x14ac:dyDescent="0.25">
@@ -9181,7 +9178,7 @@
         <v>192</v>
       </c>
       <c r="K310" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="311" spans="2:12" x14ac:dyDescent="0.25">
@@ -9209,7 +9206,7 @@
     </row>
     <row r="312" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B312" s="4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="D312" s="3" t="s">
         <v>245</v>
@@ -9227,7 +9224,7 @@
         <v>44</v>
       </c>
       <c r="K312" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="313" spans="2:12" x14ac:dyDescent="0.25">
@@ -9267,10 +9264,10 @@
         <v>248</v>
       </c>
       <c r="I314" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K314" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="315" spans="2:12" x14ac:dyDescent="0.25">
@@ -9291,7 +9288,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K315" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="316" spans="2:12" x14ac:dyDescent="0.25">
@@ -9334,10 +9331,10 @@
         <v>184</v>
       </c>
       <c r="J317" s="3" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="K317" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="318" spans="2:12" x14ac:dyDescent="0.25">
@@ -9359,7 +9356,7 @@
     </row>
     <row r="319" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B319" s="4" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D319" s="3" t="s">
         <v>245</v>
@@ -9377,7 +9374,7 @@
         <v>44</v>
       </c>
       <c r="K319" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="320" spans="2:12" x14ac:dyDescent="0.25">
@@ -9417,10 +9414,10 @@
         <v>248</v>
       </c>
       <c r="I321" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K321" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="322" spans="2:12" x14ac:dyDescent="0.25">
@@ -9441,7 +9438,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K322" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="323" spans="2:12" x14ac:dyDescent="0.25">
@@ -9484,7 +9481,7 @@
         <v>193</v>
       </c>
       <c r="K324" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="325" spans="2:12" x14ac:dyDescent="0.25">
@@ -9506,7 +9503,7 @@
     </row>
     <row r="326" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B326" s="4" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="D326" s="3" t="s">
         <v>245</v>
@@ -9524,7 +9521,7 @@
         <v>44</v>
       </c>
       <c r="K326" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="327" spans="2:12" x14ac:dyDescent="0.25">
@@ -9564,10 +9561,10 @@
         <v>248</v>
       </c>
       <c r="I328" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K328" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="329" spans="2:12" x14ac:dyDescent="0.25">
@@ -9588,7 +9585,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K329" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="330" spans="2:12" x14ac:dyDescent="0.25">
@@ -9631,7 +9628,7 @@
         <v>185</v>
       </c>
       <c r="K331" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="332" spans="2:12" x14ac:dyDescent="0.25">
@@ -9653,7 +9650,7 @@
     </row>
     <row r="333" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B333" s="4" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="D333" s="3" t="s">
         <v>245</v>
@@ -9671,7 +9668,7 @@
         <v>44</v>
       </c>
       <c r="K333" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="334" spans="2:12" x14ac:dyDescent="0.25">
@@ -9711,10 +9708,10 @@
         <v>248</v>
       </c>
       <c r="I335" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K335" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="336" spans="2:12" x14ac:dyDescent="0.25">
@@ -9735,7 +9732,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K336" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="337" spans="2:12" x14ac:dyDescent="0.25">
@@ -9778,7 +9775,7 @@
         <v>194</v>
       </c>
       <c r="K338" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="339" spans="2:12" x14ac:dyDescent="0.25">
@@ -9800,7 +9797,7 @@
     </row>
     <row r="340" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B340" s="4" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="D340" s="3" t="s">
         <v>245</v>
@@ -9818,7 +9815,7 @@
         <v>44</v>
       </c>
       <c r="K340" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="341" spans="2:12" x14ac:dyDescent="0.25">
@@ -9858,10 +9855,10 @@
         <v>248</v>
       </c>
       <c r="I342" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K342" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="343" spans="2:12" x14ac:dyDescent="0.25">
@@ -9882,7 +9879,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K343" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="344" spans="2:12" x14ac:dyDescent="0.25">
@@ -9925,7 +9922,7 @@
         <v>198</v>
       </c>
       <c r="K345" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="346" spans="2:12" x14ac:dyDescent="0.25">
@@ -9947,7 +9944,7 @@
     </row>
     <row r="347" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B347" s="4" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="D347" s="3" t="s">
         <v>245</v>
@@ -9965,7 +9962,7 @@
         <v>44</v>
       </c>
       <c r="K347" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="348" spans="2:12" x14ac:dyDescent="0.25">
@@ -10005,10 +10002,10 @@
         <v>248</v>
       </c>
       <c r="I349" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K349" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="350" spans="2:12" x14ac:dyDescent="0.25">
@@ -10029,7 +10026,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K350" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="351" spans="2:12" x14ac:dyDescent="0.25">
@@ -10072,7 +10069,7 @@
         <v>199</v>
       </c>
       <c r="K352" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="353" spans="2:12" x14ac:dyDescent="0.25">
@@ -10094,7 +10091,7 @@
     </row>
     <row r="354" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B354" s="4" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="D354" s="3" t="s">
         <v>245</v>
@@ -10112,7 +10109,7 @@
         <v>44</v>
       </c>
       <c r="K354" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="355" spans="2:12" x14ac:dyDescent="0.25">
@@ -10152,10 +10149,10 @@
         <v>248</v>
       </c>
       <c r="I356" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K356" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="357" spans="2:12" x14ac:dyDescent="0.25">
@@ -10176,7 +10173,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K357" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="358" spans="2:12" x14ac:dyDescent="0.25">
@@ -10219,7 +10216,7 @@
         <v>248</v>
       </c>
       <c r="I359" s="4" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="360" spans="2:12" x14ac:dyDescent="0.25">
@@ -10230,7 +10227,7 @@
         <v>293</v>
       </c>
       <c r="F360" s="3" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G360" s="3" t="s">
         <v>179</v>
@@ -10239,7 +10236,7 @@
         <v>195</v>
       </c>
       <c r="K360" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="361" spans="2:12" x14ac:dyDescent="0.25">
@@ -10267,7 +10264,7 @@
     </row>
     <row r="362" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B362" s="4" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D362" s="3" t="s">
         <v>245</v>
@@ -10285,7 +10282,7 @@
         <v>44</v>
       </c>
       <c r="K362" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="363" spans="2:12" x14ac:dyDescent="0.25">
@@ -10325,10 +10322,10 @@
         <v>248</v>
       </c>
       <c r="I364" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K364" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="365" spans="2:12" x14ac:dyDescent="0.25">
@@ -10349,7 +10346,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K365" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="366" spans="2:12" x14ac:dyDescent="0.25">
@@ -10392,7 +10389,7 @@
         <v>248</v>
       </c>
       <c r="I367" s="4" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="368" spans="2:12" x14ac:dyDescent="0.25">
@@ -10403,7 +10400,7 @@
         <v>293</v>
       </c>
       <c r="F368" s="3" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G368" s="3" t="s">
         <v>179</v>
@@ -10412,7 +10409,7 @@
         <v>196</v>
       </c>
       <c r="K368" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="369" spans="1:12" x14ac:dyDescent="0.25">
@@ -10440,7 +10437,7 @@
     </row>
     <row r="370" spans="1:12" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B370" s="4" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="D370" s="3" t="s">
         <v>245</v>
@@ -10458,7 +10455,7 @@
         <v>44</v>
       </c>
       <c r="K370" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="371" spans="1:12" x14ac:dyDescent="0.25">
@@ -10498,10 +10495,10 @@
         <v>248</v>
       </c>
       <c r="I372" s="4" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="K372" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="373" spans="1:12" x14ac:dyDescent="0.25">
@@ -10522,7 +10519,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K373" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="374" spans="1:12" x14ac:dyDescent="0.25">
@@ -10565,7 +10562,7 @@
         <v>248</v>
       </c>
       <c r="I375" s="4" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="376" spans="1:12" x14ac:dyDescent="0.25">
@@ -10576,7 +10573,7 @@
         <v>293</v>
       </c>
       <c r="F376" s="3" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G376" s="3" t="s">
         <v>179</v>
@@ -10585,7 +10582,7 @@
         <v>197</v>
       </c>
       <c r="K376" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="377" spans="1:12" x14ac:dyDescent="0.25">
@@ -10613,16 +10610,16 @@
     </row>
     <row r="378" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A378" s="6" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B378" s="4" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="D378" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E378" s="3" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="F378" s="3" t="s">
         <v>269</v>
@@ -10634,7 +10631,7 @@
         <v>10</v>
       </c>
       <c r="K378" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="379" spans="1:12" x14ac:dyDescent="0.25">
@@ -10660,7 +10657,7 @@
       <c r="A380" s="3"/>
       <c r="B380" s="3"/>
       <c r="E380" s="3" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="F380" s="3" t="s">
         <v>247</v>
@@ -10672,13 +10669,13 @@
         <v>248</v>
       </c>
       <c r="I380" s="4" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="J380" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L380" s="3" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="381" spans="1:12" x14ac:dyDescent="0.25">
@@ -10698,7 +10695,7 @@
         <v>46</v>
       </c>
       <c r="K381" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="382" spans="1:12" x14ac:dyDescent="0.25">
@@ -10718,7 +10715,7 @@
         <v>49</v>
       </c>
       <c r="J382" s="3" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="383" spans="1:12" x14ac:dyDescent="0.25">
@@ -10740,7 +10737,7 @@
     </row>
     <row r="384" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B384" s="4" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="D384" s="3" t="s">
         <v>245</v>
@@ -10758,7 +10755,7 @@
         <v>10</v>
       </c>
       <c r="K384" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="385" spans="2:12" x14ac:dyDescent="0.25">
@@ -10798,7 +10795,7 @@
         <v>46</v>
       </c>
       <c r="K386" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="387" spans="2:12" x14ac:dyDescent="0.25">
@@ -10819,7 +10816,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K387" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="388" spans="2:12" x14ac:dyDescent="0.25">
@@ -10862,10 +10859,10 @@
         <v>61</v>
       </c>
       <c r="J389" s="3" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="K389" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="390" spans="2:12" x14ac:dyDescent="0.25">
@@ -10887,7 +10884,7 @@
     </row>
     <row r="391" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B391" s="4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="D391" s="3" t="s">
         <v>245</v>
@@ -10905,7 +10902,7 @@
         <v>10</v>
       </c>
       <c r="K391" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="392" spans="2:12" x14ac:dyDescent="0.25">
@@ -10922,7 +10919,7 @@
         <v>248</v>
       </c>
       <c r="I392" s="4" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="J392" s="3" t="s">
         <v>289</v>
@@ -10945,7 +10942,7 @@
         <v>46</v>
       </c>
       <c r="K393" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="394" spans="2:12" x14ac:dyDescent="0.25">
@@ -10966,7 +10963,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K394" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="395" spans="2:12" x14ac:dyDescent="0.25">
@@ -11009,7 +11006,7 @@
         <v>79</v>
       </c>
       <c r="K396" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="397" spans="2:12" x14ac:dyDescent="0.25">
@@ -11065,7 +11062,7 @@
     </row>
     <row r="400" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B400" s="4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="D400" s="3" t="s">
         <v>245</v>
@@ -11083,7 +11080,7 @@
         <v>10</v>
       </c>
       <c r="K400" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="401" spans="2:12" x14ac:dyDescent="0.25">
@@ -11123,7 +11120,7 @@
         <v>46</v>
       </c>
       <c r="K402" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="403" spans="2:12" x14ac:dyDescent="0.25">
@@ -11144,7 +11141,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K403" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="404" spans="2:12" x14ac:dyDescent="0.25">
@@ -11187,7 +11184,7 @@
         <v>53</v>
       </c>
       <c r="K405" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="406" spans="2:12" x14ac:dyDescent="0.25">
@@ -11209,7 +11206,7 @@
     </row>
     <row r="407" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B407" s="4" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="D407" s="3" t="s">
         <v>245</v>
@@ -11227,7 +11224,7 @@
         <v>10</v>
       </c>
       <c r="K407" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="408" spans="2:12" x14ac:dyDescent="0.25">
@@ -11267,7 +11264,7 @@
         <v>46</v>
       </c>
       <c r="K409" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="410" spans="2:12" x14ac:dyDescent="0.25">
@@ -11288,7 +11285,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K410" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="411" spans="2:12" x14ac:dyDescent="0.25">
@@ -11331,7 +11328,7 @@
         <v>83</v>
       </c>
       <c r="K412" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="413" spans="2:12" x14ac:dyDescent="0.25">
@@ -11353,7 +11350,7 @@
     </row>
     <row r="414" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B414" s="4" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="D414" s="3" t="s">
         <v>245</v>
@@ -11371,7 +11368,7 @@
         <v>10</v>
       </c>
       <c r="K414" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="415" spans="2:12" x14ac:dyDescent="0.25">
@@ -11411,7 +11408,7 @@
         <v>46</v>
       </c>
       <c r="K416" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="417" spans="1:12" x14ac:dyDescent="0.25">
@@ -11432,7 +11429,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K417" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="418" spans="1:12" x14ac:dyDescent="0.25">
@@ -11475,7 +11472,7 @@
         <v>82</v>
       </c>
       <c r="K419" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="420" spans="1:12" x14ac:dyDescent="0.25">
@@ -11497,7 +11494,7 @@
     </row>
     <row r="421" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B421" s="4" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="D421" s="3" t="s">
         <v>325</v>
@@ -11519,7 +11516,7 @@
         <v>OMOP Primary Dx Episode</v>
       </c>
       <c r="K421" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="422" spans="1:12" x14ac:dyDescent="0.25">
@@ -11540,7 +11537,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K422" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="423" spans="1:12" x14ac:dyDescent="0.25">
@@ -11568,7 +11565,7 @@
     </row>
     <row r="424" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B424" s="4" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D424" s="3" t="s">
         <v>325</v>
@@ -11590,7 +11587,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K424" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="425" spans="1:12" x14ac:dyDescent="0.25">
@@ -11611,7 +11608,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K425" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="426" spans="1:12" x14ac:dyDescent="0.25">
@@ -11639,7 +11636,7 @@
     </row>
     <row r="427" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B427" s="4" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="G427" s="3" t="s">
         <v>39</v>
@@ -11674,19 +11671,19 @@
     </row>
     <row r="431" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A431" s="6" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="B431" s="4" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="D431" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E431" s="3" t="s">
         <v>248</v>
       </c>
       <c r="F431" s="3" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="G431" s="3" t="s">
         <v>200</v>
@@ -11699,10 +11696,10 @@
       <c r="A432" s="3"/>
       <c r="B432" s="3"/>
       <c r="D432" s="3" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="E432" s="3" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="F432" s="3" t="s">
         <v>268</v>
@@ -11714,12 +11711,12 @@
         <v>201</v>
       </c>
       <c r="K432" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="433" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E433" s="3" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="F433" s="3" t="s">
         <v>247</v>
@@ -11731,18 +11728,18 @@
         <v>248</v>
       </c>
       <c r="I433" s="4" t="s">
+        <v>684</v>
+      </c>
+      <c r="J433" s="3" t="s">
         <v>685</v>
       </c>
-      <c r="J433" s="3" t="s">
+      <c r="L433" s="3" t="s">
         <v>686</v>
-      </c>
-      <c r="L433" s="3" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="434" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E434" s="3" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="F434" s="3" t="s">
         <v>298</v>
@@ -11754,12 +11751,12 @@
         <v>204</v>
       </c>
       <c r="K434" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="435" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E435" s="3" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="F435" s="3" t="s">
         <v>298</v>
@@ -11772,12 +11769,12 @@
       </c>
       <c r="I435" s="9"/>
       <c r="K435" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="436" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B436" s="4" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D436" s="3" t="s">
         <v>245</v>
@@ -11795,7 +11792,7 @@
         <v>201</v>
       </c>
       <c r="K436" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="437" spans="2:12" x14ac:dyDescent="0.25">
@@ -11812,13 +11809,13 @@
         <v>248</v>
       </c>
       <c r="I437" s="4" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="J437" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L437" s="3" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="438" spans="2:12" x14ac:dyDescent="0.25">
@@ -11835,7 +11832,7 @@
         <v>204</v>
       </c>
       <c r="K438" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="439" spans="2:12" x14ac:dyDescent="0.25">
@@ -11870,13 +11867,13 @@
         <v>248</v>
       </c>
       <c r="I440" s="4" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="J440" s="3" t="s">
         <v>267</v>
       </c>
       <c r="L440" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="441" spans="2:12" x14ac:dyDescent="0.25">
@@ -11893,7 +11890,7 @@
         <v>206</v>
       </c>
       <c r="K441" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="442" spans="2:12" x14ac:dyDescent="0.25">
@@ -11912,7 +11909,7 @@
     </row>
     <row r="443" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B443" s="4" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="D443" s="3" t="s">
         <v>245</v>
@@ -11930,7 +11927,7 @@
         <v>201</v>
       </c>
       <c r="K443" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="444" spans="2:12" x14ac:dyDescent="0.25">
@@ -11947,13 +11944,13 @@
         <v>248</v>
       </c>
       <c r="I444" s="4" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="J444" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L444" s="3" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="445" spans="2:12" x14ac:dyDescent="0.25">
@@ -11970,7 +11967,7 @@
         <v>208</v>
       </c>
       <c r="K445" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="446" spans="2:12" x14ac:dyDescent="0.25">
@@ -11991,7 +11988,7 @@
         <v>OMOP Follow Up Visit Occurrence</v>
       </c>
       <c r="K446" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="447" spans="2:12" x14ac:dyDescent="0.25">
@@ -12008,13 +12005,13 @@
         <v>248</v>
       </c>
       <c r="I447" s="4" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="J447" s="3" t="s">
         <v>267</v>
       </c>
       <c r="L447" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="448" spans="2:12" x14ac:dyDescent="0.25">
@@ -12031,7 +12028,7 @@
         <v>207</v>
       </c>
       <c r="K448" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="449" spans="1:12" x14ac:dyDescent="0.25">
@@ -12050,7 +12047,7 @@
     </row>
     <row r="450" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B450" s="4" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="D450" s="3" t="s">
         <v>245</v>
@@ -12068,7 +12065,7 @@
         <v>201</v>
       </c>
       <c r="K450" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="451" spans="1:12" x14ac:dyDescent="0.25">
@@ -12108,7 +12105,7 @@
         <v>208</v>
       </c>
       <c r="K452" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="453" spans="1:12" x14ac:dyDescent="0.25">
@@ -12129,7 +12126,7 @@
         <v>OMOP Follow Up Visit Occurrence</v>
       </c>
       <c r="K453" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="454" spans="1:12" x14ac:dyDescent="0.25">
@@ -12146,13 +12143,13 @@
         <v>248</v>
       </c>
       <c r="I454" s="4" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="J454" s="3" t="s">
         <v>267</v>
       </c>
       <c r="L454" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="455" spans="1:12" x14ac:dyDescent="0.25">
@@ -12169,10 +12166,10 @@
         <v>210</v>
       </c>
       <c r="J455" s="3" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="K455" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="456" spans="1:12" x14ac:dyDescent="0.25">
@@ -12191,7 +12188,7 @@
     </row>
     <row r="457" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B457" s="4" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="G457" s="3" t="s">
         <v>200</v>
@@ -12202,10 +12199,10 @@
     </row>
     <row r="458" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A458" s="6" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="B458" s="4" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="D458" s="3" t="s">
         <v>255</v>
@@ -12214,7 +12211,7 @@
         <v>328</v>
       </c>
       <c r="F458" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G458" s="3" t="s">
         <v>16</v>
@@ -12223,7 +12220,7 @@
         <v>9</v>
       </c>
       <c r="K458" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="459" spans="1:12" x14ac:dyDescent="0.25">
@@ -12263,7 +12260,7 @@
         <v>212</v>
       </c>
       <c r="K460" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="461" spans="1:12" x14ac:dyDescent="0.25">
@@ -12280,7 +12277,7 @@
         <v>213</v>
       </c>
       <c r="K461" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="462" spans="1:12" x14ac:dyDescent="0.25">
@@ -12308,7 +12305,7 @@
     </row>
     <row r="463" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B463" s="4" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="D463" s="3" t="s">
         <v>255</v>
@@ -12317,7 +12314,7 @@
         <v>328</v>
       </c>
       <c r="F463" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G463" s="3" t="s">
         <v>16</v>
@@ -12326,7 +12323,7 @@
         <v>9</v>
       </c>
       <c r="K463" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="464" spans="1:12" x14ac:dyDescent="0.25">
@@ -12366,7 +12363,7 @@
         <v>212</v>
       </c>
       <c r="K465" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="466" spans="2:12" x14ac:dyDescent="0.25">
@@ -12383,7 +12380,7 @@
         <v>214</v>
       </c>
       <c r="K466" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="467" spans="2:12" x14ac:dyDescent="0.25">
@@ -12411,7 +12408,7 @@
     </row>
     <row r="468" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B468" s="4" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="D468" s="3" t="s">
         <v>255</v>
@@ -12420,7 +12417,7 @@
         <v>328</v>
       </c>
       <c r="F468" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G468" s="3" t="s">
         <v>16</v>
@@ -12429,7 +12426,7 @@
         <v>9</v>
       </c>
       <c r="K468" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="469" spans="2:12" x14ac:dyDescent="0.25">
@@ -12469,7 +12466,7 @@
         <v>212</v>
       </c>
       <c r="K470" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="471" spans="2:12" x14ac:dyDescent="0.25">
@@ -12486,7 +12483,7 @@
         <v>215</v>
       </c>
       <c r="K471" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="472" spans="2:12" x14ac:dyDescent="0.25">
@@ -12514,7 +12511,7 @@
     </row>
     <row r="473" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B473" s="4" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="D473" s="3" t="s">
         <v>255</v>
@@ -12523,7 +12520,7 @@
         <v>328</v>
       </c>
       <c r="F473" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G473" s="3" t="s">
         <v>16</v>
@@ -12532,7 +12529,7 @@
         <v>9</v>
       </c>
       <c r="K473" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="474" spans="2:12" x14ac:dyDescent="0.25">
@@ -12572,7 +12569,7 @@
         <v>212</v>
       </c>
       <c r="K475" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="476" spans="2:12" x14ac:dyDescent="0.25">
@@ -12589,7 +12586,7 @@
         <v>216</v>
       </c>
       <c r="K476" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="477" spans="2:12" x14ac:dyDescent="0.25">
@@ -12631,7 +12628,7 @@
     </row>
     <row r="479" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B479" s="4" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D479" s="3" t="s">
         <v>255</v>
@@ -12640,7 +12637,7 @@
         <v>328</v>
       </c>
       <c r="F479" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G479" s="3" t="s">
         <v>16</v>
@@ -12649,7 +12646,7 @@
         <v>9</v>
       </c>
       <c r="K479" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="480" spans="2:12" x14ac:dyDescent="0.25">
@@ -12689,7 +12686,7 @@
         <v>212</v>
       </c>
       <c r="K481" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="482" spans="1:12" x14ac:dyDescent="0.25">
@@ -12706,12 +12703,12 @@
         <v>220</v>
       </c>
       <c r="K482" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="483" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B483" s="4" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D483" s="3" t="s">
         <v>255</v>
@@ -12720,7 +12717,7 @@
         <v>328</v>
       </c>
       <c r="F483" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G483" s="3" t="s">
         <v>16</v>
@@ -12729,7 +12726,7 @@
         <v>9</v>
       </c>
       <c r="K483" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="484" spans="1:12" x14ac:dyDescent="0.25">
@@ -12769,7 +12766,7 @@
         <v>212</v>
       </c>
       <c r="K485" s="3" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="486" spans="1:12" x14ac:dyDescent="0.25">
@@ -12786,12 +12783,12 @@
         <v>221</v>
       </c>
       <c r="K486" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="487" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B487" s="4" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="G487" s="3" t="s">
         <v>211</v>
@@ -12818,10 +12815,10 @@
     </row>
     <row r="490" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A490" s="6" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B490" s="4" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="D490" s="3" t="s">
         <v>245</v>
@@ -12830,7 +12827,7 @@
         <v>287</v>
       </c>
       <c r="F490" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G490" s="3" t="s">
         <v>16</v>
@@ -12839,7 +12836,7 @@
         <v>9</v>
       </c>
       <c r="K490" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="491" spans="1:12" x14ac:dyDescent="0.25">
@@ -12879,7 +12876,7 @@
         <v>233</v>
       </c>
       <c r="K492" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="493" spans="1:12" x14ac:dyDescent="0.25">
@@ -12898,7 +12895,7 @@
     </row>
     <row r="494" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B494" s="4" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="D494" s="3" t="s">
         <v>245</v>
@@ -12907,7 +12904,7 @@
         <v>287</v>
       </c>
       <c r="F494" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G494" s="3" t="s">
         <v>16</v>
@@ -12916,7 +12913,7 @@
         <v>9</v>
       </c>
       <c r="K494" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="495" spans="1:12" x14ac:dyDescent="0.25">
@@ -12933,13 +12930,13 @@
         <v>248</v>
       </c>
       <c r="I495" s="4" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="J495" s="3" t="s">
         <v>289</v>
       </c>
       <c r="L495" s="3" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
     </row>
     <row r="496" spans="1:12" x14ac:dyDescent="0.25">
@@ -12947,7 +12944,7 @@
         <v>343</v>
       </c>
       <c r="F496" s="3" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="G496" s="3" t="s">
         <v>16</v>
@@ -12960,7 +12957,7 @@
         <v>OMOP Tobacco Smoking Status Observation</v>
       </c>
       <c r="K496" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="497" spans="1:12" x14ac:dyDescent="0.25">
@@ -13000,12 +12997,12 @@
         <v>235</v>
       </c>
       <c r="K498" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="499" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B499" s="4" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="D499" s="3" t="s">
         <v>245</v>
@@ -13014,7 +13011,7 @@
         <v>287</v>
       </c>
       <c r="F499" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G499" s="3" t="s">
         <v>16</v>
@@ -13023,7 +13020,7 @@
         <v>9</v>
       </c>
       <c r="K499" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="500" spans="1:12" x14ac:dyDescent="0.25">
@@ -13054,7 +13051,7 @@
         <v>343</v>
       </c>
       <c r="F501" s="3" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="G501" s="3" t="s">
         <v>16</v>
@@ -13067,7 +13064,7 @@
         <v>OMOP Tobacco Smoking Status Observation</v>
       </c>
       <c r="K501" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="502" spans="1:12" x14ac:dyDescent="0.25">
@@ -13107,7 +13104,7 @@
         <v>248</v>
       </c>
       <c r="I503" s="4" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="504" spans="1:12" x14ac:dyDescent="0.25">
@@ -13115,7 +13112,7 @@
         <v>293</v>
       </c>
       <c r="F504" s="3" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="G504" s="3" t="s">
         <v>232</v>
@@ -13124,24 +13121,24 @@
         <v>234</v>
       </c>
       <c r="K504" s="3" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="505" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A505" s="6" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="B505" s="4" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="D505" s="3" t="s">
         <v>260</v>
       </c>
       <c r="E505" s="3" t="s">
-        <v>545</v>
+        <v>304</v>
       </c>
       <c r="F505" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G505" s="3" t="s">
         <v>16</v>
@@ -13186,7 +13183,7 @@
         <v>312</v>
       </c>
       <c r="F508" s="3" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="G508" s="3" t="s">
         <v>225</v>
@@ -13211,7 +13208,7 @@
     </row>
     <row r="510" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E510" s="3" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="F510" s="3" t="s">
         <v>269</v>
@@ -13225,7 +13222,7 @@
     </row>
     <row r="511" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B511" s="4" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="D511" s="3" t="s">
         <v>255</v>
@@ -13234,7 +13231,7 @@
         <v>328</v>
       </c>
       <c r="F511" s="3" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G511" s="3" t="s">
         <v>16</v>
@@ -13274,7 +13271,7 @@
         <v>225</v>
       </c>
       <c r="H513" s="6" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="I513" s="4" t="str">
         <f>$B$505</f>
@@ -13331,10 +13328,10 @@
     </row>
     <row r="517" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B517" s="4" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="C517" s="3" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="G517" s="13" t="s">
         <v>225</v>
@@ -13359,7 +13356,7 @@
     </row>
     <row r="523" spans="2:10" ht="27" x14ac:dyDescent="0.25">
       <c r="B523" s="4" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="G523" s="13" t="s">
         <v>7</v>

</xml_diff>